<commit_message>
Test_case Excel Updated CMS to SMS
</commit_message>
<xml_diff>
--- a/testing/Test_cases.xlsx
+++ b/testing/Test_cases.xlsx
@@ -14,7 +14,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="184">
   <si>
-    <t>CMS Testing Summary</t>
+    <t>SMS Testing Summary</t>
   </si>
   <si>
     <t>By Test Level</t>
@@ -648,10 +648,10 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -1025,7 +1025,7 @@
       <c r="I2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="7">
+      <c r="J2" s="8">
         <v>46218.0</v>
       </c>
       <c r="K2" s="6" t="s">
@@ -1063,7 +1063,7 @@
       <c r="I3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="7">
+      <c r="J3" s="8">
         <v>46218.0</v>
       </c>
       <c r="K3" s="6" t="s">
@@ -1101,7 +1101,7 @@
       <c r="I4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="J4" s="7">
+      <c r="J4" s="8">
         <v>46219.0</v>
       </c>
       <c r="K4" s="6" t="s">
@@ -1139,7 +1139,7 @@
       <c r="I5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="J5" s="7">
+      <c r="J5" s="8">
         <v>46219.0</v>
       </c>
       <c r="K5" s="6" t="s">
@@ -1177,7 +1177,7 @@
       <c r="I6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="J6" s="7">
+      <c r="J6" s="8">
         <v>46220.0</v>
       </c>
       <c r="K6" s="6" t="s">
@@ -1215,7 +1215,7 @@
       <c r="I7" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="J7" s="7">
+      <c r="J7" s="8">
         <v>46220.0</v>
       </c>
       <c r="K7" s="6" t="s">
@@ -1851,15 +1851,15 @@
       <c r="B6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="7">
         <f>COUNTIF(Sheet1!B$2:B1000, B6)</f>
         <v>6</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="7">
         <f>COUNTIFS(Sheet1!B$2:B1000, B6, Sheet1!I$2:I1000, "Pass")</f>
         <v>5</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="7">
         <f>COUNTIFS(Sheet1!B$2:B1000, B6, Sheet1!I$2:I1000, "Fail")</f>
         <v>1</v>
       </c>
@@ -1872,15 +1872,15 @@
       <c r="B7" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="7">
         <f>COUNTIF(Sheet1!B$2:B1000, B7)</f>
         <v>5</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="7">
         <f>COUNTIFS(Sheet1!B$2:B1000, B7, Sheet1!I$2:I1000, "Pass")</f>
         <v>4</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="7">
         <f>COUNTIFS(Sheet1!B$2:B1000, B7, Sheet1!I$2:I1000, "Fail")</f>
         <v>1</v>
       </c>
@@ -1893,15 +1893,15 @@
       <c r="B8" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="7">
         <f>COUNTIF(Sheet1!B$2:B1000, B8)</f>
         <v>5</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="7">
         <f>COUNTIFS(Sheet1!B$2:B1000, B8, Sheet1!I$2:I1000, "Pass")</f>
         <v>4</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="7">
         <f>COUNTIFS(Sheet1!B$2:B1000, B8, Sheet1!I$2:I1000, "Fail")</f>
         <v>1</v>
       </c>
@@ -1914,15 +1914,15 @@
       <c r="B9" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="7">
         <f>COUNTIF(Sheet1!B$2:B1000, B9)</f>
         <v>5</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="7">
         <f>COUNTIFS(Sheet1!B$2:B1000, B9, Sheet1!I$2:I1000, "Pass")</f>
         <v>4</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="7">
         <f>COUNTIFS(Sheet1!B$2:B1000, B9, Sheet1!I$2:I1000, "Fail")</f>
         <v>1</v>
       </c>
@@ -1935,15 +1935,15 @@
       <c r="B10" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="7">
         <f t="shared" ref="C10:E10" si="2">SUM(C6:C9)</f>
         <v>21</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="7">
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="7">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>

</xml_diff>